<commit_message>
Perform some function in Excel which is very usfull to take decision
</commit_message>
<xml_diff>
--- a/customer_purchase_dataseet.xlsx
+++ b/customer_purchase_dataseet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Project\Fashion Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC11DE6-43EF-4C91-9E3C-34BC735988CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{970D09CD-A2AD-45B9-A1D7-83FBD0218A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{52086F29-C266-4FF4-89C2-E090B5B922C7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{52086F29-C266-4FF4-89C2-E090B5B922C7}"/>
   </bookViews>
   <sheets>
     <sheet name="customer_purchase_dataset" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="18" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11202" uniqueCount="2143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11208" uniqueCount="2145">
   <si>
     <t>Customer ID</t>
   </si>
@@ -6489,6 +6489,12 @@
   </si>
   <si>
     <t>Sum of Quantity</t>
+  </si>
+  <si>
+    <t>Avg customer Rating</t>
+  </si>
+  <si>
+    <t>Count Order Status</t>
   </si>
 </sst>
 </file>
@@ -6631,7 +6637,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6823,6 +6829,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -6999,7 +7017,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
@@ -7009,7 +7027,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -29673,7 +29695,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9C4D9EC7-27AC-4348-A21E-DBA9539076F5}" name="PivotTable6" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9C4D9EC7-27AC-4348-A21E-DBA9539076F5}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="N4:O8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="19">
     <pivotField showAll="0"/>
@@ -30313,7 +30335,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BD666DC8-D823-4A2E-B9D6-744E8CECD67F}" name="PivotTable5" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BD666DC8-D823-4A2E-B9D6-744E8CECD67F}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="K4:L13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="19">
     <pivotField showAll="0"/>
@@ -31250,7 +31272,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9EFD4469-6190-47E2-BA15-958C600D53B4}" name="PivotTable4" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9EFD4469-6190-47E2-BA15-958C600D53B4}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="H4:I25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="19">
     <pivotField showAll="0"/>
@@ -31943,7 +31965,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3ACB998A-7630-4A83-BD8B-1B28DC473487}" name="PivotTable3" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3ACB998A-7630-4A83-BD8B-1B28DC473487}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E4:F20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="19">
     <pivotField showAll="0"/>
@@ -32611,7 +32633,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2CBE7931-D42A-4061-B2BF-518C4E91979A}" name="PivotTable1" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2CBE7931-D42A-4061-B2BF-518C4E91979A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B4:C298" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="19">
     <pivotField showAll="0"/>
@@ -94562,7 +94584,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC577DC6-4E57-4A33-8AF9-49E64330F658}">
-  <dimension ref="A2:U7"/>
+  <dimension ref="A2:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
@@ -94583,9 +94605,12 @@
     <col min="16" max="16" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -94635,7 +94660,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>54</v>
       </c>
@@ -94685,14 +94710,23 @@
       <c r="P3" s="4">
         <v>4</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3" s="1" t="s">
         <v>2136</v>
       </c>
-      <c r="U3" t="s">
+      <c r="U3" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="W3" s="1" t="s">
+        <v>2143</v>
+      </c>
+      <c r="Y3" s="7" t="s">
+        <v>2144</v>
+      </c>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="7"/>
+      <c r="AB3" s="7"/>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>448</v>
       </c>
@@ -94742,16 +94776,32 @@
       <c r="P4" s="4">
         <v>0</v>
       </c>
-      <c r="S4">
+      <c r="S4" s="4">
         <f>SUM(customer_purchase_dataset!J2:J1201)</f>
         <v>1487</v>
       </c>
-      <c r="U4">
+      <c r="U4" s="4">
         <f>SUM(customer_purchase_dataset!L2:L1201)</f>
         <v>1162625.0399999989</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="W4" s="4">
+        <f>ROUND(AVERAGE(customer_purchase_dataset!P2:P1201),2)</f>
+        <v>3.58</v>
+      </c>
+      <c r="Y4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z4" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA4" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="AB4" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>749</v>
       </c>
@@ -94801,8 +94851,21 @@
       <c r="P5" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y5" s="9" cm="1">
+        <f t="array" ref="Y5:AB5">COUNTIFS(customer_purchase_dataset!O2:O1201,Summery!Y4:AB4)</f>
+        <v>694</v>
+      </c>
+      <c r="Z5" s="9">
+        <v>180</v>
+      </c>
+      <c r="AA5" s="9">
+        <v>158</v>
+      </c>
+      <c r="AB5" s="9">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>1484</v>
       </c>
@@ -94853,7 +94916,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>1914</v>
       </c>
@@ -94905,6 +94968,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="Y3:AB3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -94996,31 +95062,31 @@
       <c r="B5" s="6" t="s">
         <v>1932</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5">
         <v>4268.7205000000004</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5">
         <v>77111.229999999981</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>544</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5">
         <v>6</v>
       </c>
       <c r="K5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L5">
         <v>142357.25999999992</v>
       </c>
       <c r="N5" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="O5" s="7">
+      <c r="O5">
         <v>36395.93</v>
       </c>
     </row>
@@ -95028,31 +95094,31 @@
       <c r="B6" s="6" t="s">
         <v>899</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6">
         <v>2983.9160000000002</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6">
         <v>94976.059999999939</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6">
         <v>35</v>
       </c>
       <c r="K6" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6">
         <v>101065.73</v>
       </c>
       <c r="N6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="O6" s="7">
+      <c r="O6">
         <v>23338.400000000001</v>
       </c>
     </row>
@@ -95060,31 +95126,31 @@
       <c r="B7" s="6" t="s">
         <v>876</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7">
         <v>616.19899999999996</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7">
         <v>82568.119999999981</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7">
         <v>45</v>
       </c>
       <c r="K7" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="L7" s="7">
+      <c r="L7">
         <v>137194.43000000002</v>
       </c>
       <c r="N7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="7">
+      <c r="O7">
         <v>35241.730000000003</v>
       </c>
     </row>
@@ -95092,31 +95158,31 @@
       <c r="B8" s="6" t="s">
         <v>543</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8">
         <v>1798.8675000000001</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8">
         <v>98794.66</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8">
         <v>45</v>
       </c>
       <c r="K8" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8">
         <v>164760.19000000009</v>
       </c>
       <c r="N8" s="6" t="s">
         <v>2138</v>
       </c>
-      <c r="O8" s="7">
+      <c r="O8">
         <v>94976.06</v>
       </c>
     </row>
@@ -95124,25 +95190,25 @@
       <c r="B9" s="6" t="s">
         <v>1404</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9">
         <v>2534.34</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9">
         <v>83449.45</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9">
         <v>26</v>
       </c>
       <c r="K9" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="L9" s="7">
+      <c r="L9">
         <v>152344.89999999991</v>
       </c>
     </row>
@@ -95150,25 +95216,25 @@
       <c r="B10" s="6" t="s">
         <v>2006</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10">
         <v>2220.36</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10">
         <v>94890.01</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10">
         <v>18</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="L10" s="7">
+      <c r="L10">
         <v>166162.22999999998</v>
       </c>
     </row>
@@ -95176,25 +95242,25 @@
       <c r="B11" s="6" t="s">
         <v>907</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11">
         <v>3850.8879999999999</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11">
         <v>83796.059999999983</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11">
         <v>42</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="7">
+      <c r="L11">
         <v>144774.39000000001</v>
       </c>
     </row>
@@ -95202,25 +95268,25 @@
       <c r="B12" s="6" t="s">
         <v>1607</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12">
         <v>3097.6205</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12">
         <v>62491.100000000006</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>743</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12">
         <v>2</v>
       </c>
       <c r="K12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="L12" s="7">
+      <c r="L12">
         <v>153965.91000000009</v>
       </c>
     </row>
@@ -95228,25 +95294,25 @@
       <c r="B13" s="6" t="s">
         <v>1967</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13">
         <v>2624.6325000000002</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13">
         <v>66495.710000000006</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13">
         <v>22</v>
       </c>
       <c r="K13" s="6" t="s">
         <v>2138</v>
       </c>
-      <c r="L13" s="7">
+      <c r="L13">
         <v>1162625.04</v>
       </c>
     </row>
@@ -95254,19 +95320,19 @@
       <c r="B14" s="6" t="s">
         <v>570</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14">
         <v>1958.6279999999999</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14">
         <v>68508.7</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14">
         <v>24</v>
       </c>
     </row>
@@ -95274,19 +95340,19 @@
       <c r="B15" s="6" t="s">
         <v>1813</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15">
         <v>4200.558</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15">
         <v>59476.370000000032</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15">
         <v>8</v>
       </c>
     </row>
@@ -95294,19 +95360,19 @@
       <c r="B16" s="6" t="s">
         <v>1207</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16">
         <v>2280.63</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16">
         <v>72316.419999999984</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16">
         <v>50</v>
       </c>
     </row>
@@ -95314,19 +95380,19 @@
       <c r="B17" s="6" t="s">
         <v>471</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17">
         <v>2361.06</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17">
         <v>78319.400000000009</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17">
         <v>6</v>
       </c>
     </row>
@@ -95334,19 +95400,19 @@
       <c r="B18" s="6" t="s">
         <v>1095</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18">
         <v>1080.0840000000001</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18">
         <v>63892.880000000005</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="I18" s="7">
+      <c r="I18">
         <v>29</v>
       </c>
     </row>
@@ -95354,19 +95420,19 @@
       <c r="B19" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19">
         <v>5180.4480000000003</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19">
         <v>75538.869999999966</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19">
         <v>12</v>
       </c>
     </row>
@@ -95374,19 +95440,19 @@
       <c r="B20" s="6" t="s">
         <v>1338</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20">
         <v>3453.4639999999999</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>2138</v>
       </c>
-      <c r="F20" s="7">
+      <c r="F20">
         <v>1162625.0399999996</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="I20" s="7">
+      <c r="I20">
         <v>20</v>
       </c>
     </row>
@@ -95394,13 +95460,13 @@
       <c r="B21" s="6" t="s">
         <v>710</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21">
         <v>1018.845</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21">
         <v>18</v>
       </c>
     </row>
@@ -95408,13 +95474,13 @@
       <c r="B22" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22">
         <v>5540.4960000000001</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I22" s="7">
+      <c r="I22">
         <v>32</v>
       </c>
     </row>
@@ -95422,13 +95488,13 @@
       <c r="B23" s="6" t="s">
         <v>1474</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23">
         <v>5679.1980000000003</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="I23" s="7">
+      <c r="I23">
         <v>33</v>
       </c>
     </row>
@@ -95436,13 +95502,13 @@
       <c r="B24" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24">
         <v>3840.48</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="I24" s="7">
+      <c r="I24">
         <v>34</v>
       </c>
     </row>
@@ -95450,13 +95516,13 @@
       <c r="B25" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25">
         <v>4393.4400000000005</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>2138</v>
       </c>
-      <c r="I25" s="7">
+      <c r="I25">
         <v>507</v>
       </c>
     </row>
@@ -95464,7 +95530,7 @@
       <c r="B26" s="6" t="s">
         <v>994</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26">
         <v>3670.0830000000001</v>
       </c>
     </row>
@@ -95472,7 +95538,7 @@
       <c r="B27" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27">
         <v>4673.2139999999999</v>
       </c>
     </row>
@@ -95480,7 +95546,7 @@
       <c r="B28" s="6" t="s">
         <v>1216</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28">
         <v>2541.0495000000001</v>
       </c>
     </row>
@@ -95488,7 +95554,7 @@
       <c r="B29" s="6" t="s">
         <v>496</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29">
         <v>1089.3375000000001</v>
       </c>
     </row>
@@ -95496,7 +95562,7 @@
       <c r="B30" s="6" t="s">
         <v>1769</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30">
         <v>4325.3549999999996</v>
       </c>
     </row>
@@ -95504,7 +95570,7 @@
       <c r="B31" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="C31" s="7">
+      <c r="C31">
         <v>3968.847999999999</v>
       </c>
     </row>
@@ -95512,7 +95578,7 @@
       <c r="B32" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="C32" s="7">
+      <c r="C32">
         <v>3862.88</v>
       </c>
     </row>
@@ -95520,7 +95586,7 @@
       <c r="B33" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="C33" s="7">
+      <c r="C33">
         <v>849.66300000000001</v>
       </c>
     </row>
@@ -95528,7 +95594,7 @@
       <c r="B34" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="C34" s="7">
+      <c r="C34">
         <v>1361.904</v>
       </c>
     </row>
@@ -95536,7 +95602,7 @@
       <c r="B35" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="C35" s="7">
+      <c r="C35">
         <v>5057.0519999999997</v>
       </c>
     </row>
@@ -95544,7 +95610,7 @@
       <c r="B36" s="6" t="s">
         <v>1161</v>
       </c>
-      <c r="C36" s="7">
+      <c r="C36">
         <v>3410.6329999999998</v>
       </c>
     </row>
@@ -95552,7 +95618,7 @@
       <c r="B37" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="C37" s="7">
+      <c r="C37">
         <v>4614.3020000000006</v>
       </c>
     </row>
@@ -95560,7 +95626,7 @@
       <c r="B38" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C38" s="7">
+      <c r="C38">
         <v>4669.0199999999995</v>
       </c>
     </row>
@@ -95568,7 +95634,7 @@
       <c r="B39" s="6" t="s">
         <v>997</v>
       </c>
-      <c r="C39" s="7">
+      <c r="C39">
         <v>1143.338</v>
       </c>
     </row>
@@ -95576,7 +95642,7 @@
       <c r="B40" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="C40" s="7">
+      <c r="C40">
         <v>2493.9899999999998</v>
       </c>
     </row>
@@ -95584,7 +95650,7 @@
       <c r="B41" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="C41" s="7">
+      <c r="C41">
         <v>3810.2999999999993</v>
       </c>
     </row>
@@ -95592,7 +95658,7 @@
       <c r="B42" s="6" t="s">
         <v>837</v>
       </c>
-      <c r="C42" s="7">
+      <c r="C42">
         <v>2459.1239999999998</v>
       </c>
     </row>
@@ -95600,7 +95666,7 @@
       <c r="B43" s="6" t="s">
         <v>861</v>
       </c>
-      <c r="C43" s="7">
+      <c r="C43">
         <v>3358.2080000000001</v>
       </c>
     </row>
@@ -95608,7 +95674,7 @@
       <c r="B44" s="6" t="s">
         <v>923</v>
       </c>
-      <c r="C44" s="7">
+      <c r="C44">
         <v>3031.7429999999999</v>
       </c>
     </row>
@@ -95616,7 +95682,7 @@
       <c r="B45" s="6" t="s">
         <v>1658</v>
       </c>
-      <c r="C45" s="7">
+      <c r="C45">
         <v>661.54499999999996</v>
       </c>
     </row>
@@ -95624,7 +95690,7 @@
       <c r="B46" s="6" t="s">
         <v>644</v>
       </c>
-      <c r="C46" s="7">
+      <c r="C46">
         <v>2335.0050000000001</v>
       </c>
     </row>
@@ -95632,7 +95698,7 @@
       <c r="B47" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="C47" s="7">
+      <c r="C47">
         <v>4653.1499999999996</v>
       </c>
     </row>
@@ -95640,7 +95706,7 @@
       <c r="B48" s="6" t="s">
         <v>1988</v>
       </c>
-      <c r="C48" s="7">
+      <c r="C48">
         <v>3033.8625000000002</v>
       </c>
     </row>
@@ -95648,7 +95714,7 @@
       <c r="B49" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="C49" s="7">
+      <c r="C49">
         <v>1524.624</v>
       </c>
     </row>
@@ -95656,7 +95722,7 @@
       <c r="B50" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C50" s="7">
+      <c r="C50">
         <v>3246.4439999999995</v>
       </c>
     </row>
@@ -95664,7 +95730,7 @@
       <c r="B51" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C51" s="7">
+      <c r="C51">
         <v>5351.5020000000004</v>
       </c>
     </row>
@@ -95672,7 +95738,7 @@
       <c r="B52" s="6" t="s">
         <v>1686</v>
       </c>
-      <c r="C52" s="7">
+      <c r="C52">
         <v>1174.884</v>
       </c>
     </row>
@@ -95680,7 +95746,7 @@
       <c r="B53" s="6" t="s">
         <v>1642</v>
       </c>
-      <c r="C53" s="7">
+      <c r="C53">
         <v>769.03</v>
       </c>
     </row>
@@ -95688,7 +95754,7 @@
       <c r="B54" s="6" t="s">
         <v>1213</v>
       </c>
-      <c r="C54" s="7">
+      <c r="C54">
         <v>2013.12</v>
       </c>
     </row>
@@ -95696,7 +95762,7 @@
       <c r="B55" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="C55" s="7">
+      <c r="C55">
         <v>3696.1999999999994</v>
       </c>
     </row>
@@ -95704,7 +95770,7 @@
       <c r="B56" s="6" t="s">
         <v>985</v>
       </c>
-      <c r="C56" s="7">
+      <c r="C56">
         <v>607.12</v>
       </c>
     </row>
@@ -95712,7 +95778,7 @@
       <c r="B57" s="6" t="s">
         <v>1504</v>
       </c>
-      <c r="C57" s="7">
+      <c r="C57">
         <v>848.23199999999997</v>
       </c>
     </row>
@@ -95720,7 +95786,7 @@
       <c r="B58" s="6" t="s">
         <v>2100</v>
       </c>
-      <c r="C58" s="7">
+      <c r="C58">
         <v>2384.3325</v>
       </c>
     </row>
@@ -95728,7 +95794,7 @@
       <c r="B59" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="C59" s="7">
+      <c r="C59">
         <v>7598.0999999999976</v>
       </c>
     </row>
@@ -95736,7 +95802,7 @@
       <c r="B60" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="C60" s="7">
+      <c r="C60">
         <v>4800.119999999999</v>
       </c>
     </row>
@@ -95744,7 +95810,7 @@
       <c r="B61" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="C61" s="7">
+      <c r="C61">
         <v>1377.624</v>
       </c>
     </row>
@@ -95752,7 +95818,7 @@
       <c r="B62" s="6" t="s">
         <v>1955</v>
       </c>
-      <c r="C62" s="7">
+      <c r="C62">
         <v>2781.5830000000001</v>
       </c>
     </row>
@@ -95760,7 +95826,7 @@
       <c r="B63" s="6" t="s">
         <v>582</v>
       </c>
-      <c r="C63" s="7">
+      <c r="C63">
         <v>4357.5280000000002</v>
       </c>
     </row>
@@ -95768,7 +95834,7 @@
       <c r="B64" s="6" t="s">
         <v>518</v>
       </c>
-      <c r="C64" s="7">
+      <c r="C64">
         <v>6310.0800000000027</v>
       </c>
     </row>
@@ -95776,7 +95842,7 @@
       <c r="B65" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="C65" s="7">
+      <c r="C65">
         <v>3260.096</v>
       </c>
     </row>
@@ -95784,7 +95850,7 @@
       <c r="B66" s="6" t="s">
         <v>562</v>
       </c>
-      <c r="C66" s="7">
+      <c r="C66">
         <v>1825.41</v>
       </c>
     </row>
@@ -95792,7 +95858,7 @@
       <c r="B67" s="6" t="s">
         <v>1890</v>
       </c>
-      <c r="C67" s="7">
+      <c r="C67">
         <v>3939.85</v>
       </c>
     </row>
@@ -95800,7 +95866,7 @@
       <c r="B68" s="6" t="s">
         <v>1393</v>
       </c>
-      <c r="C68" s="7">
+      <c r="C68">
         <v>2337.84</v>
       </c>
     </row>
@@ -95808,7 +95874,7 @@
       <c r="B69" s="6" t="s">
         <v>1156</v>
       </c>
-      <c r="C69" s="7">
+      <c r="C69">
         <v>1331.7429999999999</v>
       </c>
     </row>
@@ -95816,7 +95882,7 @@
       <c r="B70" s="6" t="s">
         <v>1928</v>
       </c>
-      <c r="C70" s="7">
+      <c r="C70">
         <v>3581.9749999999999</v>
       </c>
     </row>
@@ -95824,7 +95890,7 @@
       <c r="B71" s="6" t="s">
         <v>1746</v>
       </c>
-      <c r="C71" s="7">
+      <c r="C71">
         <v>3583.17</v>
       </c>
     </row>
@@ -95832,7 +95898,7 @@
       <c r="B72" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="C72" s="7">
+      <c r="C72">
         <v>1753.04</v>
       </c>
     </row>
@@ -95840,7 +95906,7 @@
       <c r="B73" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="C73" s="7">
+      <c r="C73">
         <v>1750.432</v>
       </c>
     </row>
@@ -95848,7 +95914,7 @@
       <c r="B74" s="6" t="s">
         <v>662</v>
       </c>
-      <c r="C74" s="7">
+      <c r="C74">
         <v>2389.4324999999999</v>
       </c>
     </row>
@@ -95856,7 +95922,7 @@
       <c r="B75" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="C75" s="7">
+      <c r="C75">
         <v>3067.038</v>
       </c>
     </row>
@@ -95864,7 +95930,7 @@
       <c r="B76" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="C76" s="7">
+      <c r="C76">
         <v>4667.25</v>
       </c>
     </row>
@@ -95872,7 +95938,7 @@
       <c r="B77" s="6" t="s">
         <v>2135</v>
       </c>
-      <c r="C77" s="7">
+      <c r="C77">
         <v>1314.2249999999999</v>
       </c>
     </row>
@@ -95880,7 +95946,7 @@
       <c r="B78" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="C78" s="7">
+      <c r="C78">
         <v>3880.32</v>
       </c>
     </row>
@@ -95888,7 +95954,7 @@
       <c r="B79" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="C79" s="7">
+      <c r="C79">
         <v>699.32</v>
       </c>
     </row>
@@ -95896,7 +95962,7 @@
       <c r="B80" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="C80" s="7">
+      <c r="C80">
         <v>4036.14</v>
       </c>
     </row>
@@ -95904,7 +95970,7 @@
       <c r="B81" s="6" t="s">
         <v>1007</v>
       </c>
-      <c r="C81" s="7">
+      <c r="C81">
         <v>4617.9399999999996</v>
       </c>
     </row>
@@ -95912,7 +95978,7 @@
       <c r="B82" s="6" t="s">
         <v>1449</v>
       </c>
-      <c r="C82" s="7">
+      <c r="C82">
         <v>2484.1</v>
       </c>
     </row>
@@ -95920,7 +95986,7 @@
       <c r="B83" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="C83" s="7">
+      <c r="C83">
         <v>4402.9439999999986</v>
       </c>
     </row>
@@ -95928,7 +95994,7 @@
       <c r="B84" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="C84" s="7">
+      <c r="C84">
         <v>6507.6959999999981</v>
       </c>
     </row>
@@ -95936,7 +96002,7 @@
       <c r="B85" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="C85" s="7">
+      <c r="C85">
         <v>3243.5185000000001</v>
       </c>
     </row>
@@ -95944,7 +96010,7 @@
       <c r="B86" s="6" t="s">
         <v>1943</v>
       </c>
-      <c r="C86" s="7">
+      <c r="C86">
         <v>2193.7860000000001</v>
       </c>
     </row>
@@ -95952,7 +96018,7 @@
       <c r="B87" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="C87" s="7">
+      <c r="C87">
         <v>2587.7550000000001</v>
       </c>
     </row>
@@ -95960,7 +96026,7 @@
       <c r="B88" s="6" t="s">
         <v>1440</v>
       </c>
-      <c r="C88" s="7">
+      <c r="C88">
         <v>5762.3580000000002</v>
       </c>
     </row>
@@ -95968,7 +96034,7 @@
       <c r="B89" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C89" s="7">
+      <c r="C89">
         <v>2748.096</v>
       </c>
     </row>
@@ -95976,7 +96042,7 @@
       <c r="B90" s="6" t="s">
         <v>963</v>
       </c>
-      <c r="C90" s="7">
+      <c r="C90">
         <v>2000.3520000000001</v>
       </c>
     </row>
@@ -95984,7 +96050,7 @@
       <c r="B91" s="6" t="s">
         <v>1695</v>
       </c>
-      <c r="C91" s="7">
+      <c r="C91">
         <v>3131.3035</v>
       </c>
     </row>
@@ -95992,7 +96058,7 @@
       <c r="B92" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="C92" s="7">
+      <c r="C92">
         <v>4525.152000000001</v>
       </c>
     </row>
@@ -96000,7 +96066,7 @@
       <c r="B93" s="6" t="s">
         <v>534</v>
       </c>
-      <c r="C93" s="7">
+      <c r="C93">
         <v>1812.9135000000001</v>
       </c>
     </row>
@@ -96008,7 +96074,7 @@
       <c r="B94" s="6" t="s">
         <v>748</v>
       </c>
-      <c r="C94" s="7">
+      <c r="C94">
         <v>1631.1479999999999</v>
       </c>
     </row>
@@ -96016,7 +96082,7 @@
       <c r="B95" s="6" t="s">
         <v>1602</v>
       </c>
-      <c r="C95" s="7">
+      <c r="C95">
         <v>3288.1995000000002</v>
       </c>
     </row>
@@ -96024,7 +96090,7 @@
       <c r="B96" s="6" t="s">
         <v>634</v>
       </c>
-      <c r="C96" s="7">
+      <c r="C96">
         <v>3444.2240000000011</v>
       </c>
     </row>
@@ -96032,7 +96098,7 @@
       <c r="B97" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="C97" s="7">
+      <c r="C97">
         <v>1622.9199999999998</v>
       </c>
     </row>
@@ -96040,7 +96106,7 @@
       <c r="B98" s="6" t="s">
         <v>1721</v>
       </c>
-      <c r="C98" s="7">
+      <c r="C98">
         <v>3558.7759999999998</v>
       </c>
     </row>
@@ -96048,7 +96114,7 @@
       <c r="B99" s="6" t="s">
         <v>2129</v>
       </c>
-      <c r="C99" s="7">
+      <c r="C99">
         <v>1895.874</v>
       </c>
     </row>
@@ -96056,7 +96122,7 @@
       <c r="B100" s="6" t="s">
         <v>696</v>
       </c>
-      <c r="C100" s="7">
+      <c r="C100">
         <v>4497.0200000000004</v>
       </c>
     </row>
@@ -96064,7 +96130,7 @@
       <c r="B101" s="6" t="s">
         <v>1252</v>
       </c>
-      <c r="C101" s="7">
+      <c r="C101">
         <v>2207.6819999999998</v>
       </c>
     </row>
@@ -96072,7 +96138,7 @@
       <c r="B102" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="C102" s="7">
+      <c r="C102">
         <v>1584.7950000000001</v>
       </c>
     </row>
@@ -96080,7 +96146,7 @@
       <c r="B103" s="6" t="s">
         <v>2067</v>
       </c>
-      <c r="C103" s="7">
+      <c r="C103">
         <v>2279.42</v>
       </c>
     </row>
@@ -96088,7 +96154,7 @@
       <c r="B104" s="6" t="s">
         <v>917</v>
       </c>
-      <c r="C104" s="7">
+      <c r="C104">
         <v>832.71100000000001</v>
       </c>
     </row>
@@ -96096,7 +96162,7 @@
       <c r="B105" s="6" t="s">
         <v>776</v>
       </c>
-      <c r="C105" s="7">
+      <c r="C105">
         <v>2443.2669999999998</v>
       </c>
     </row>
@@ -96104,7 +96170,7 @@
       <c r="B106" s="6" t="s">
         <v>950</v>
       </c>
-      <c r="C106" s="7">
+      <c r="C106">
         <v>1179.4090000000001</v>
       </c>
     </row>
@@ -96112,7 +96178,7 @@
       <c r="B107" s="6" t="s">
         <v>1358</v>
       </c>
-      <c r="C107" s="7">
+      <c r="C107">
         <v>2732.7089999999998</v>
       </c>
     </row>
@@ -96120,7 +96186,7 @@
       <c r="B108" s="6" t="s">
         <v>1166</v>
       </c>
-      <c r="C108" s="7">
+      <c r="C108">
         <v>2114.5279999999998</v>
       </c>
     </row>
@@ -96128,7 +96194,7 @@
       <c r="B109" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="C109" s="7">
+      <c r="C109">
         <v>3802.0449999999992</v>
       </c>
     </row>
@@ -96136,7 +96202,7 @@
       <c r="B110" s="6" t="s">
         <v>864</v>
       </c>
-      <c r="C110" s="7">
+      <c r="C110">
         <v>824.14</v>
       </c>
     </row>
@@ -96144,7 +96210,7 @@
       <c r="B111" s="6" t="s">
         <v>1193</v>
       </c>
-      <c r="C111" s="7">
+      <c r="C111">
         <v>4026.61</v>
       </c>
     </row>
@@ -96152,7 +96218,7 @@
       <c r="B112" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="C112" s="7">
+      <c r="C112">
         <v>3862.2000000000007</v>
       </c>
     </row>
@@ -96160,7 +96226,7 @@
       <c r="B113" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="C113" s="7">
+      <c r="C113">
         <v>3564.0480000000002</v>
       </c>
     </row>
@@ -96168,7 +96234,7 @@
       <c r="B114" s="6" t="s">
         <v>1714</v>
       </c>
-      <c r="C114" s="7">
+      <c r="C114">
         <v>1238.8720000000001</v>
       </c>
     </row>
@@ -96176,7 +96242,7 @@
       <c r="B115" s="6" t="s">
         <v>1567</v>
       </c>
-      <c r="C115" s="7">
+      <c r="C115">
         <v>3924.0630000000001</v>
       </c>
     </row>
@@ -96184,7 +96250,7 @@
       <c r="B116" s="6" t="s">
         <v>2044</v>
       </c>
-      <c r="C116" s="7">
+      <c r="C116">
         <v>2403.9839999999999</v>
       </c>
     </row>
@@ -96192,7 +96258,7 @@
       <c r="B117" s="6" t="s">
         <v>1680</v>
       </c>
-      <c r="C117" s="7">
+      <c r="C117">
         <v>3179.8020000000001</v>
       </c>
     </row>
@@ -96200,7 +96266,7 @@
       <c r="B118" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="C118" s="7">
+      <c r="C118">
         <v>6192.1600000000017</v>
       </c>
     </row>
@@ -96208,7 +96274,7 @@
       <c r="B119" s="6" t="s">
         <v>1356</v>
       </c>
-      <c r="C119" s="7">
+      <c r="C119">
         <v>2055.7109999999998</v>
       </c>
     </row>
@@ -96216,7 +96282,7 @@
       <c r="B120" s="6" t="s">
         <v>1029</v>
       </c>
-      <c r="C120" s="7">
+      <c r="C120">
         <v>2879.2080000000001</v>
       </c>
     </row>
@@ -96224,7 +96290,7 @@
       <c r="B121" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="C121" s="7">
+      <c r="C121">
         <v>5399.91</v>
       </c>
     </row>
@@ -96232,7 +96298,7 @@
       <c r="B122" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C122" s="7">
+      <c r="C122">
         <v>4861.1499999999987</v>
       </c>
     </row>
@@ -96240,7 +96306,7 @@
       <c r="B123" s="6" t="s">
         <v>1859</v>
       </c>
-      <c r="C123" s="7">
+      <c r="C123">
         <v>600.96</v>
       </c>
     </row>
@@ -96248,7 +96314,7 @@
       <c r="B124" s="6" t="s">
         <v>1949</v>
       </c>
-      <c r="C124" s="7">
+      <c r="C124">
         <v>2210.8440000000001</v>
       </c>
     </row>
@@ -96256,7 +96322,7 @@
       <c r="B125" s="6" t="s">
         <v>1159</v>
       </c>
-      <c r="C125" s="7">
+      <c r="C125">
         <v>3895.3325</v>
       </c>
     </row>
@@ -96264,7 +96330,7 @@
       <c r="B126" s="6" t="s">
         <v>935</v>
       </c>
-      <c r="C126" s="7">
+      <c r="C126">
         <v>1162.43</v>
       </c>
     </row>
@@ -96272,7 +96338,7 @@
       <c r="B127" s="6" t="s">
         <v>2077</v>
       </c>
-      <c r="C127" s="7">
+      <c r="C127">
         <v>2004.6075000000001</v>
       </c>
     </row>
@@ -96280,7 +96346,7 @@
       <c r="B128" s="6" t="s">
         <v>773</v>
       </c>
-      <c r="C128" s="7">
+      <c r="C128">
         <v>2595.5909999999999</v>
       </c>
     </row>
@@ -96288,7 +96354,7 @@
       <c r="B129" s="6" t="s">
         <v>1350</v>
       </c>
-      <c r="C129" s="7">
+      <c r="C129">
         <v>3473.3425000000002</v>
       </c>
     </row>
@@ -96296,7 +96362,7 @@
       <c r="B130" s="6" t="s">
         <v>742</v>
       </c>
-      <c r="C130" s="7">
+      <c r="C130">
         <v>1644.3979999999999</v>
       </c>
     </row>
@@ -96304,7 +96370,7 @@
       <c r="B131" s="6" t="s">
         <v>801</v>
       </c>
-      <c r="C131" s="7">
+      <c r="C131">
         <v>2650.4850000000001</v>
       </c>
     </row>
@@ -96312,7 +96378,7 @@
       <c r="B132" s="6" t="s">
         <v>614</v>
       </c>
-      <c r="C132" s="7">
+      <c r="C132">
         <v>4825.8339999999998</v>
       </c>
     </row>
@@ -96320,7 +96386,7 @@
       <c r="B133" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C133" s="7">
+      <c r="C133">
         <v>4121.1280000000006</v>
       </c>
     </row>
@@ -96328,7 +96394,7 @@
       <c r="B134" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="C134" s="7">
+      <c r="C134">
         <v>5663.36</v>
       </c>
     </row>
@@ -96336,7 +96402,7 @@
       <c r="B135" s="6" t="s">
         <v>1846</v>
       </c>
-      <c r="C135" s="7">
+      <c r="C135">
         <v>3059.0479999999998</v>
       </c>
     </row>
@@ -96344,7 +96410,7 @@
       <c r="B136" s="6" t="s">
         <v>1308</v>
       </c>
-      <c r="C136" s="7">
+      <c r="C136">
         <v>564.851</v>
       </c>
     </row>
@@ -96352,7 +96418,7 @@
       <c r="B137" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="C137" s="7">
+      <c r="C137">
         <v>2209.1199999999994</v>
       </c>
     </row>
@@ -96360,7 +96426,7 @@
       <c r="B138" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="C138" s="7">
+      <c r="C138">
         <v>4430.41</v>
       </c>
     </row>
@@ -96368,7 +96434,7 @@
       <c r="B139" s="6" t="s">
         <v>1249</v>
       </c>
-      <c r="C139" s="7">
+      <c r="C139">
         <v>822.39599999999996</v>
       </c>
     </row>
@@ -96376,7 +96442,7 @@
       <c r="B140" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="C140" s="7">
+      <c r="C140">
         <v>706.34699999999998</v>
       </c>
     </row>
@@ -96384,7 +96450,7 @@
       <c r="B141" s="6" t="s">
         <v>1574</v>
       </c>
-      <c r="C141" s="7">
+      <c r="C141">
         <v>1311.3969999999999</v>
       </c>
     </row>
@@ -96392,7 +96458,7 @@
       <c r="B142" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="C142" s="7">
+      <c r="C142">
         <v>3737.369999999999</v>
       </c>
     </row>
@@ -96400,7 +96466,7 @@
       <c r="B143" s="6" t="s">
         <v>1589</v>
       </c>
-      <c r="C143" s="7">
+      <c r="C143">
         <v>1873.155</v>
       </c>
     </row>
@@ -96408,7 +96474,7 @@
       <c r="B144" s="6" t="s">
         <v>2060</v>
       </c>
-      <c r="C144" s="7">
+      <c r="C144">
         <v>2064.1149999999998</v>
       </c>
     </row>
@@ -96416,7 +96482,7 @@
       <c r="B145" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="C145" s="7">
+      <c r="C145">
         <v>3969.6360000000004</v>
       </c>
     </row>
@@ -96424,7 +96490,7 @@
       <c r="B146" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C146" s="7">
+      <c r="C146">
         <v>4205.4799999999996</v>
       </c>
     </row>
@@ -96432,7 +96498,7 @@
       <c r="B147" s="6" t="s">
         <v>1639</v>
       </c>
-      <c r="C147" s="7">
+      <c r="C147">
         <v>2636.6745000000001</v>
       </c>
     </row>
@@ -96440,7 +96506,7 @@
       <c r="B148" s="6" t="s">
         <v>1921</v>
       </c>
-      <c r="C148" s="7">
+      <c r="C148">
         <v>1952.93</v>
       </c>
     </row>
@@ -96448,7 +96514,7 @@
       <c r="B149" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="C149" s="7">
+      <c r="C149">
         <v>3104.6719999999996</v>
       </c>
     </row>
@@ -96456,7 +96522,7 @@
       <c r="B150" s="6" t="s">
         <v>1751</v>
       </c>
-      <c r="C150" s="7">
+      <c r="C150">
         <v>2490.9639999999999</v>
       </c>
     </row>
@@ -96464,7 +96530,7 @@
       <c r="B151" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="C151" s="7">
+      <c r="C151">
         <v>3631.7360000000017</v>
       </c>
     </row>
@@ -96472,7 +96538,7 @@
       <c r="B152" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C152" s="7">
+      <c r="C152">
         <v>1982.2800000000004</v>
       </c>
     </row>
@@ -96480,7 +96546,7 @@
       <c r="B153" s="6" t="s">
         <v>2089</v>
       </c>
-      <c r="C153" s="7">
+      <c r="C153">
         <v>4374.7</v>
       </c>
     </row>
@@ -96488,7 +96554,7 @@
       <c r="B154" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="C154" s="7">
+      <c r="C154">
         <v>3251.3799999999997</v>
       </c>
     </row>
@@ -96496,7 +96562,7 @@
       <c r="B155" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="C155" s="7">
+      <c r="C155">
         <v>3836.547</v>
       </c>
     </row>
@@ -96504,7 +96570,7 @@
       <c r="B156" s="6" t="s">
         <v>1120</v>
       </c>
-      <c r="C156" s="7">
+      <c r="C156">
         <v>1743.4059999999999</v>
       </c>
     </row>
@@ -96512,7 +96578,7 @@
       <c r="B157" s="6" t="s">
         <v>2086</v>
       </c>
-      <c r="C157" s="7">
+      <c r="C157">
         <v>1559.4390000000001</v>
       </c>
     </row>
@@ -96520,7 +96586,7 @@
       <c r="B158" s="6" t="s">
         <v>991</v>
       </c>
-      <c r="C158" s="7">
+      <c r="C158">
         <v>1114.152</v>
       </c>
     </row>
@@ -96528,7 +96594,7 @@
       <c r="B159" s="6" t="s">
         <v>688</v>
       </c>
-      <c r="C159" s="7">
+      <c r="C159">
         <v>4828.47</v>
       </c>
     </row>
@@ -96536,7 +96602,7 @@
       <c r="B160" s="6" t="s">
         <v>639</v>
       </c>
-      <c r="C160" s="7">
+      <c r="C160">
         <v>2474.808</v>
       </c>
     </row>
@@ -96544,7 +96610,7 @@
       <c r="B161" s="6" t="s">
         <v>2009</v>
       </c>
-      <c r="C161" s="7">
+      <c r="C161">
         <v>1351.28</v>
       </c>
     </row>
@@ -96552,7 +96618,7 @@
       <c r="B162" s="6" t="s">
         <v>2049</v>
       </c>
-      <c r="C162" s="7">
+      <c r="C162">
         <v>2399.7674999999999</v>
       </c>
     </row>
@@ -96560,7 +96626,7 @@
       <c r="B163" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="C163" s="7">
+      <c r="C163">
         <v>2974.7339999999999</v>
       </c>
     </row>
@@ -96568,7 +96634,7 @@
       <c r="B164" s="6" t="s">
         <v>1617</v>
       </c>
-      <c r="C164" s="7">
+      <c r="C164">
         <v>712.94500000000005</v>
       </c>
     </row>
@@ -96576,7 +96642,7 @@
       <c r="B165" s="6" t="s">
         <v>1556</v>
       </c>
-      <c r="C165" s="7">
+      <c r="C165">
         <v>723.95699999999999</v>
       </c>
     </row>
@@ -96584,7 +96650,7 @@
       <c r="B166" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C166" s="7">
+      <c r="C166">
         <v>2576.7000000000007</v>
       </c>
     </row>
@@ -96592,7 +96658,7 @@
       <c r="B167" s="6" t="s">
         <v>1370</v>
       </c>
-      <c r="C167" s="7">
+      <c r="C167">
         <v>1490.874</v>
       </c>
     </row>
@@ -96600,7 +96666,7 @@
       <c r="B168" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="C168" s="7">
+      <c r="C168">
         <v>4405.5719999999992</v>
       </c>
     </row>
@@ -96608,7 +96674,7 @@
       <c r="B169" s="6" t="s">
         <v>1935</v>
       </c>
-      <c r="C169" s="7">
+      <c r="C169">
         <v>2820.5515</v>
       </c>
     </row>
@@ -96616,7 +96682,7 @@
       <c r="B170" s="6" t="s">
         <v>765</v>
       </c>
-      <c r="C170" s="7">
+      <c r="C170">
         <v>4582.4160000000002</v>
       </c>
     </row>
@@ -96624,7 +96690,7 @@
       <c r="B171" s="6" t="s">
         <v>1903</v>
       </c>
-      <c r="C171" s="7">
+      <c r="C171">
         <v>1124.739</v>
       </c>
     </row>
@@ -96632,7 +96698,7 @@
       <c r="B172" s="6" t="s">
         <v>1710</v>
       </c>
-      <c r="C172" s="7">
+      <c r="C172">
         <v>3214.96</v>
       </c>
     </row>
@@ -96640,7 +96706,7 @@
       <c r="B173" s="6" t="s">
         <v>2014</v>
       </c>
-      <c r="C173" s="7">
+      <c r="C173">
         <v>1801.932</v>
       </c>
     </row>
@@ -96648,7 +96714,7 @@
       <c r="B174" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="C174" s="7">
+      <c r="C174">
         <v>5624.8319999999994</v>
       </c>
     </row>
@@ -96656,7 +96722,7 @@
       <c r="B175" s="6" t="s">
         <v>1793</v>
       </c>
-      <c r="C175" s="7">
+      <c r="C175">
         <v>1235.9849999999999</v>
       </c>
     </row>
@@ -96664,7 +96730,7 @@
       <c r="B176" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C176" s="7">
+      <c r="C176">
         <v>3774.2320000000013</v>
       </c>
     </row>
@@ -96672,7 +96738,7 @@
       <c r="B177" s="6" t="s">
         <v>1135</v>
       </c>
-      <c r="C177" s="7">
+      <c r="C177">
         <v>2343.627</v>
       </c>
     </row>
@@ -96680,7 +96746,7 @@
       <c r="B178" s="6" t="s">
         <v>2002</v>
       </c>
-      <c r="C178" s="7">
+      <c r="C178">
         <v>2400.5120000000002</v>
       </c>
     </row>
@@ -96688,7 +96754,7 @@
       <c r="B179" s="6" t="s">
         <v>809</v>
       </c>
-      <c r="C179" s="7">
+      <c r="C179">
         <v>5776.7</v>
       </c>
     </row>
@@ -96696,7 +96762,7 @@
       <c r="B180" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C180" s="7">
+      <c r="C180">
         <v>2285.4960000000001</v>
       </c>
     </row>
@@ -96704,7 +96770,7 @@
       <c r="B181" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="C181" s="7">
+      <c r="C181">
         <v>1469.0840000000001</v>
       </c>
     </row>
@@ -96712,7 +96778,7 @@
       <c r="B182" s="6" t="s">
         <v>1905</v>
       </c>
-      <c r="C182" s="7">
+      <c r="C182">
         <v>2660.9335000000001</v>
       </c>
     </row>
@@ -96720,7 +96786,7 @@
       <c r="B183" s="6" t="s">
         <v>1869</v>
       </c>
-      <c r="C183" s="7">
+      <c r="C183">
         <v>783.33500000000004</v>
       </c>
     </row>
@@ -96728,7 +96794,7 @@
       <c r="B184" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="C184" s="7">
+      <c r="C184">
         <v>835.34400000000005</v>
       </c>
     </row>
@@ -96736,7 +96802,7 @@
       <c r="B185" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="C185" s="7">
+      <c r="C185">
         <v>2981.61</v>
       </c>
     </row>
@@ -96744,7 +96810,7 @@
       <c r="B186" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C186" s="7">
+      <c r="C186">
         <v>6808.1944999999978</v>
       </c>
     </row>
@@ -96752,7 +96818,7 @@
       <c r="B187" s="6" t="s">
         <v>1841</v>
       </c>
-      <c r="C187" s="7">
+      <c r="C187">
         <v>548.33399999999995</v>
       </c>
     </row>
@@ -96760,7 +96826,7 @@
       <c r="B188" s="6" t="s">
         <v>594</v>
       </c>
-      <c r="C188" s="7">
+      <c r="C188">
         <v>2832.22</v>
       </c>
     </row>
@@ -96768,7 +96834,7 @@
       <c r="B189" s="6" t="s">
         <v>694</v>
       </c>
-      <c r="C189" s="7">
+      <c r="C189">
         <v>2084.8000000000002</v>
       </c>
     </row>
@@ -96776,7 +96842,7 @@
       <c r="B190" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C190" s="7">
+      <c r="C190">
         <v>2156.2399999999998</v>
       </c>
     </row>
@@ -96784,7 +96850,7 @@
       <c r="B191" s="6" t="s">
         <v>1997</v>
       </c>
-      <c r="C191" s="7">
+      <c r="C191">
         <v>3416.2240000000002</v>
       </c>
     </row>
@@ -96792,7 +96858,7 @@
       <c r="B192" s="6" t="s">
         <v>713</v>
       </c>
-      <c r="C192" s="7">
+      <c r="C192">
         <v>1843.88</v>
       </c>
     </row>
@@ -96800,7 +96866,7 @@
       <c r="B193" s="6" t="s">
         <v>1605</v>
       </c>
-      <c r="C193" s="7">
+      <c r="C193">
         <v>3187.585</v>
       </c>
     </row>
@@ -96808,7 +96874,7 @@
       <c r="B194" s="6" t="s">
         <v>1430</v>
       </c>
-      <c r="C194" s="7">
+      <c r="C194">
         <v>775.91499999999996</v>
       </c>
     </row>
@@ -96816,7 +96882,7 @@
       <c r="B195" s="6" t="s">
         <v>2011</v>
       </c>
-      <c r="C195" s="7">
+      <c r="C195">
         <v>1028.6510000000001</v>
       </c>
     </row>
@@ -96824,7 +96890,7 @@
       <c r="B196" s="6" t="s">
         <v>1756</v>
       </c>
-      <c r="C196" s="7">
+      <c r="C196">
         <v>1792.7349999999999</v>
       </c>
     </row>
@@ -96832,7 +96898,7 @@
       <c r="B197" s="6" t="s">
         <v>2123</v>
       </c>
-      <c r="C197" s="7">
+      <c r="C197">
         <v>887.83500000000004</v>
       </c>
     </row>
@@ -96840,7 +96906,7 @@
       <c r="B198" s="6" t="s">
         <v>516</v>
       </c>
-      <c r="C198" s="7">
+      <c r="C198">
         <v>2780.0239999999999</v>
       </c>
     </row>
@@ -96848,7 +96914,7 @@
       <c r="B199" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="C199" s="7">
+      <c r="C199">
         <v>10886.911999999995</v>
       </c>
     </row>
@@ -96856,7 +96922,7 @@
       <c r="B200" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="C200" s="7">
+      <c r="C200">
         <v>2854.5499999999997</v>
       </c>
     </row>
@@ -96864,7 +96930,7 @@
       <c r="B201" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="C201" s="7">
+      <c r="C201">
         <v>2189.232</v>
       </c>
     </row>
@@ -96872,7 +96938,7 @@
       <c r="B202" s="6" t="s">
         <v>468</v>
       </c>
-      <c r="C202" s="7">
+      <c r="C202">
         <v>4702.9320000000007</v>
       </c>
     </row>
@@ -96880,7 +96946,7 @@
       <c r="B203" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C203" s="7">
+      <c r="C203">
         <v>4493.8789999999999</v>
       </c>
     </row>
@@ -96888,7 +96954,7 @@
       <c r="B204" s="6" t="s">
         <v>1240</v>
       </c>
-      <c r="C204" s="7">
+      <c r="C204">
         <v>1661.1479999999999</v>
       </c>
     </row>
@@ -96896,7 +96962,7 @@
       <c r="B205" s="6" t="s">
         <v>557</v>
       </c>
-      <c r="C205" s="7">
+      <c r="C205">
         <v>5980.2</v>
       </c>
     </row>
@@ -96904,7 +96970,7 @@
       <c r="B206" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="C206" s="7">
+      <c r="C206">
         <v>5603.8799999999983</v>
       </c>
     </row>
@@ -96912,7 +96978,7 @@
       <c r="B207" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="C207" s="7">
+      <c r="C207">
         <v>756.22500000000002</v>
       </c>
     </row>
@@ -96920,7 +96986,7 @@
       <c r="B208" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="C208" s="7">
+      <c r="C208">
         <v>1146.8309999999999</v>
       </c>
     </row>
@@ -96928,7 +96994,7 @@
       <c r="B209" s="6" t="s">
         <v>880</v>
       </c>
-      <c r="C209" s="7">
+      <c r="C209">
         <v>2555.13</v>
       </c>
     </row>
@@ -96936,7 +97002,7 @@
       <c r="B210" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="C210" s="7">
+      <c r="C210">
         <v>3183.7439999999997</v>
       </c>
     </row>
@@ -96944,7 +97010,7 @@
       <c r="B211" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="C211" s="7">
+      <c r="C211">
         <v>4433.1570000000002</v>
       </c>
     </row>
@@ -96952,7 +97018,7 @@
       <c r="B212" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="C212" s="7">
+      <c r="C212">
         <v>3333.5400000000004</v>
       </c>
     </row>
@@ -96960,7 +97026,7 @@
       <c r="B213" s="6" t="s">
         <v>700</v>
       </c>
-      <c r="C213" s="7">
+      <c r="C213">
         <v>2030.825</v>
       </c>
     </row>
@@ -96968,7 +97034,7 @@
       <c r="B214" s="6" t="s">
         <v>560</v>
       </c>
-      <c r="C214" s="7">
+      <c r="C214">
         <v>3199.6964999999996</v>
       </c>
     </row>
@@ -96976,7 +97042,7 @@
       <c r="B215" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="C215" s="7">
+      <c r="C215">
         <v>889.16200000000003</v>
       </c>
     </row>
@@ -96984,7 +97050,7 @@
       <c r="B216" s="6" t="s">
         <v>618</v>
       </c>
-      <c r="C216" s="7">
+      <c r="C216">
         <v>1671.4559999999999</v>
       </c>
     </row>
@@ -96992,7 +97058,7 @@
       <c r="B217" s="6" t="s">
         <v>756</v>
       </c>
-      <c r="C217" s="7">
+      <c r="C217">
         <v>3823.362000000001</v>
       </c>
     </row>
@@ -97000,7 +97066,7 @@
       <c r="B218" s="6" t="s">
         <v>893</v>
       </c>
-      <c r="C218" s="7">
+      <c r="C218">
         <v>970.24</v>
       </c>
     </row>
@@ -97008,7 +97074,7 @@
       <c r="B219" s="6" t="s">
         <v>1244</v>
       </c>
-      <c r="C219" s="7">
+      <c r="C219">
         <v>3473.3649999999998</v>
       </c>
     </row>
@@ -97016,7 +97082,7 @@
       <c r="B220" s="6" t="s">
         <v>493</v>
       </c>
-      <c r="C220" s="7">
+      <c r="C220">
         <v>3894.7814999999991</v>
       </c>
     </row>
@@ -97024,7 +97090,7 @@
       <c r="B221" s="6" t="s">
         <v>2056</v>
       </c>
-      <c r="C221" s="7">
+      <c r="C221">
         <v>3856.212</v>
       </c>
     </row>
@@ -97032,7 +97098,7 @@
       <c r="B222" s="6" t="s">
         <v>1419</v>
       </c>
-      <c r="C222" s="7">
+      <c r="C222">
         <v>665.62800000000004</v>
       </c>
     </row>
@@ -97040,7 +97106,7 @@
       <c r="B223" s="6" t="s">
         <v>1615</v>
       </c>
-      <c r="C223" s="7">
+      <c r="C223">
         <v>682.43200000000002</v>
       </c>
     </row>
@@ -97048,7 +97114,7 @@
       <c r="B224" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="C224" s="7">
+      <c r="C224">
         <v>868.70399999999995</v>
       </c>
     </row>
@@ -97056,7 +97122,7 @@
       <c r="B225" s="6" t="s">
         <v>670</v>
       </c>
-      <c r="C225" s="7">
+      <c r="C225">
         <v>804.28499999999997</v>
       </c>
     </row>
@@ -97064,7 +97130,7 @@
       <c r="B226" s="6" t="s">
         <v>1336</v>
       </c>
-      <c r="C226" s="7">
+      <c r="C226">
         <v>3287.837</v>
       </c>
     </row>
@@ -97072,7 +97138,7 @@
       <c r="B227" s="6" t="s">
         <v>1098</v>
       </c>
-      <c r="C227" s="7">
+      <c r="C227">
         <v>2531.0400000000004</v>
       </c>
     </row>
@@ -97080,7 +97146,7 @@
       <c r="B228" s="6" t="s">
         <v>530</v>
       </c>
-      <c r="C228" s="7">
+      <c r="C228">
         <v>4236.9840000000004</v>
       </c>
     </row>
@@ -97088,7 +97154,7 @@
       <c r="B229" s="6" t="s">
         <v>1002</v>
       </c>
-      <c r="C229" s="7">
+      <c r="C229">
         <v>889.3</v>
       </c>
     </row>
@@ -97096,7 +97162,7 @@
       <c r="B230" s="6" t="s">
         <v>760</v>
       </c>
-      <c r="C230" s="7">
+      <c r="C230">
         <v>2248.232</v>
       </c>
     </row>
@@ -97104,7 +97170,7 @@
       <c r="B231" s="6" t="s">
         <v>461</v>
       </c>
-      <c r="C231" s="7">
+      <c r="C231">
         <v>1731.1999999999998</v>
       </c>
     </row>
@@ -97112,7 +97178,7 @@
       <c r="B232" s="6" t="s">
         <v>1610</v>
       </c>
-      <c r="C232" s="7">
+      <c r="C232">
         <v>1867.7284999999999</v>
       </c>
     </row>
@@ -97120,7 +97186,7 @@
       <c r="B233" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="C233" s="7">
+      <c r="C233">
         <v>5513.7879999999996</v>
       </c>
     </row>
@@ -97128,7 +97194,7 @@
       <c r="B234" s="6" t="s">
         <v>826</v>
       </c>
-      <c r="C234" s="7">
+      <c r="C234">
         <v>1075.992</v>
       </c>
     </row>
@@ -97136,7 +97202,7 @@
       <c r="B235" s="6" t="s">
         <v>1591</v>
       </c>
-      <c r="C235" s="7">
+      <c r="C235">
         <v>500.57</v>
       </c>
     </row>
@@ -97144,7 +97210,7 @@
       <c r="B236" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="C236" s="7">
+      <c r="C236">
         <v>2934.0359999999996</v>
       </c>
     </row>
@@ -97152,7 +97218,7 @@
       <c r="B237" s="6" t="s">
         <v>842</v>
       </c>
-      <c r="C237" s="7">
+      <c r="C237">
         <v>1716.1200000000001</v>
       </c>
     </row>
@@ -97160,7 +97226,7 @@
       <c r="B238" s="6" t="s">
         <v>1139</v>
       </c>
-      <c r="C238" s="7">
+      <c r="C238">
         <v>2173.5360000000001</v>
       </c>
     </row>
@@ -97168,7 +97234,7 @@
       <c r="B239" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="C239" s="7">
+      <c r="C239">
         <v>2462.5549999999998</v>
       </c>
     </row>
@@ -97176,7 +97242,7 @@
       <c r="B240" s="6" t="s">
         <v>551</v>
       </c>
-      <c r="C240" s="7">
+      <c r="C240">
         <v>2246.3040000000001</v>
       </c>
     </row>
@@ -97184,7 +97250,7 @@
       <c r="B241" s="6" t="s">
         <v>1797</v>
       </c>
-      <c r="C241" s="7">
+      <c r="C241">
         <v>684.91200000000003</v>
       </c>
     </row>
@@ -97192,7 +97258,7 @@
       <c r="B242" s="6" t="s">
         <v>1856</v>
       </c>
-      <c r="C242" s="7">
+      <c r="C242">
         <v>3078.9679999999998</v>
       </c>
     </row>
@@ -97200,7 +97266,7 @@
       <c r="B243" s="6" t="s">
         <v>429</v>
       </c>
-      <c r="C243" s="7">
+      <c r="C243">
         <v>3897.8940000000011</v>
       </c>
     </row>
@@ -97208,7 +97274,7 @@
       <c r="B244" s="6" t="s">
         <v>1169</v>
       </c>
-      <c r="C244" s="7">
+      <c r="C244">
         <v>3655.2159999999999</v>
       </c>
     </row>
@@ -97216,7 +97282,7 @@
       <c r="B245" s="6" t="s">
         <v>1053</v>
       </c>
-      <c r="C245" s="7">
+      <c r="C245">
         <v>1555.096</v>
       </c>
     </row>
@@ -97224,7 +97290,7 @@
       <c r="B246" s="6" t="s">
         <v>1743</v>
       </c>
-      <c r="C246" s="7">
+      <c r="C246">
         <v>2284.36</v>
       </c>
     </row>
@@ -97232,7 +97298,7 @@
       <c r="B247" s="6" t="s">
         <v>2079</v>
       </c>
-      <c r="C247" s="7">
+      <c r="C247">
         <v>1772.2260000000001</v>
       </c>
     </row>
@@ -97240,7 +97306,7 @@
       <c r="B248" s="6" t="s">
         <v>1085</v>
       </c>
-      <c r="C248" s="7">
+      <c r="C248">
         <v>2102.4450000000002</v>
       </c>
     </row>
@@ -97248,7 +97314,7 @@
       <c r="B249" s="6" t="s">
         <v>931</v>
       </c>
-      <c r="C249" s="7">
+      <c r="C249">
         <v>2279.0340000000001</v>
       </c>
     </row>
@@ -97256,7 +97322,7 @@
       <c r="B250" s="6" t="s">
         <v>979</v>
       </c>
-      <c r="C250" s="7">
+      <c r="C250">
         <v>1830.069</v>
       </c>
     </row>
@@ -97264,7 +97330,7 @@
       <c r="B251" s="6" t="s">
         <v>1470</v>
       </c>
-      <c r="C251" s="7">
+      <c r="C251">
         <v>3916.8539999999998</v>
       </c>
     </row>
@@ -97272,7 +97338,7 @@
       <c r="B252" s="6" t="s">
         <v>913</v>
       </c>
-      <c r="C252" s="7">
+      <c r="C252">
         <v>2321.527</v>
       </c>
     </row>
@@ -97280,7 +97346,7 @@
       <c r="B253" s="6" t="s">
         <v>512</v>
       </c>
-      <c r="C253" s="7">
+      <c r="C253">
         <v>4013.56</v>
       </c>
     </row>
@@ -97288,7 +97354,7 @@
       <c r="B254" s="6" t="s">
         <v>958</v>
       </c>
-      <c r="C254" s="7">
+      <c r="C254">
         <v>2259.1239999999998</v>
       </c>
     </row>
@@ -97296,7 +97362,7 @@
       <c r="B255" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C255" s="7">
+      <c r="C255">
         <v>3939.1199999999994</v>
       </c>
     </row>
@@ -97304,7 +97370,7 @@
       <c r="B256" s="6" t="s">
         <v>505</v>
       </c>
-      <c r="C256" s="7">
+      <c r="C256">
         <v>3774.92</v>
       </c>
     </row>
@@ -97312,7 +97378,7 @@
       <c r="B257" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C257" s="7">
+      <c r="C257">
         <v>6475.2149999999974</v>
       </c>
     </row>
@@ -97320,7 +97386,7 @@
       <c r="B258" s="6" t="s">
         <v>819</v>
       </c>
-      <c r="C258" s="7">
+      <c r="C258">
         <v>5684.94</v>
       </c>
     </row>
@@ -97328,7 +97394,7 @@
       <c r="B259" s="6" t="s">
         <v>591</v>
       </c>
-      <c r="C259" s="7">
+      <c r="C259">
         <v>4608.4499999999989</v>
       </c>
     </row>
@@ -97336,7 +97402,7 @@
       <c r="B260" s="6" t="s">
         <v>2040</v>
       </c>
-      <c r="C260" s="7">
+      <c r="C260">
         <v>969.85699999999997</v>
       </c>
     </row>
@@ -97344,7 +97410,7 @@
       <c r="B261" s="6" t="s">
         <v>1352</v>
       </c>
-      <c r="C261" s="7">
+      <c r="C261">
         <v>3694.8989999999999</v>
       </c>
     </row>
@@ -97352,7 +97418,7 @@
       <c r="B262" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="C262" s="7">
+      <c r="C262">
         <v>2733.9569999999994</v>
       </c>
     </row>
@@ -97360,7 +97426,7 @@
       <c r="B263" s="6" t="s">
         <v>1633</v>
       </c>
-      <c r="C263" s="7">
+      <c r="C263">
         <v>1261.1880000000001</v>
       </c>
     </row>
@@ -97368,7 +97434,7 @@
       <c r="B264" s="6" t="s">
         <v>1832</v>
       </c>
-      <c r="C264" s="7">
+      <c r="C264">
         <v>537.16650000000004</v>
       </c>
     </row>
@@ -97376,7 +97442,7 @@
       <c r="B265" s="6" t="s">
         <v>2091</v>
       </c>
-      <c r="C265" s="7">
+      <c r="C265">
         <v>2531.7719999999999</v>
       </c>
     </row>
@@ -97384,7 +97450,7 @@
       <c r="B266" s="6" t="s">
         <v>911</v>
       </c>
-      <c r="C266" s="7">
+      <c r="C266">
         <v>1693.6075000000001</v>
       </c>
     </row>
@@ -97392,7 +97458,7 @@
       <c r="B267" s="6" t="s">
         <v>1864</v>
       </c>
-      <c r="C267" s="7">
+      <c r="C267">
         <v>2310.942</v>
       </c>
     </row>
@@ -97400,7 +97466,7 @@
       <c r="B268" s="6" t="s">
         <v>1790</v>
       </c>
-      <c r="C268" s="7">
+      <c r="C268">
         <v>3205.433</v>
       </c>
     </row>
@@ -97408,7 +97474,7 @@
       <c r="B269" s="6" t="s">
         <v>1490</v>
       </c>
-      <c r="C269" s="7">
+      <c r="C269">
         <v>1184.1310000000001</v>
       </c>
     </row>
@@ -97416,7 +97482,7 @@
       <c r="B270" s="6" t="s">
         <v>1873</v>
       </c>
-      <c r="C270" s="7">
+      <c r="C270">
         <v>5901.8249999999998</v>
       </c>
     </row>
@@ -97424,7 +97490,7 @@
       <c r="B271" s="6" t="s">
         <v>1519</v>
       </c>
-      <c r="C271" s="7">
+      <c r="C271">
         <v>2737.3964999999998</v>
       </c>
     </row>
@@ -97432,7 +97498,7 @@
       <c r="B272" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C272" s="7">
+      <c r="C272">
         <v>5729.8149999999996</v>
       </c>
     </row>
@@ -97440,7 +97506,7 @@
       <c r="B273" s="6" t="s">
         <v>1178</v>
       </c>
-      <c r="C273" s="7">
+      <c r="C273">
         <v>763.66</v>
       </c>
     </row>
@@ -97448,7 +97514,7 @@
       <c r="B274" s="6" t="s">
         <v>961</v>
       </c>
-      <c r="C274" s="7">
+      <c r="C274">
         <v>549.19600000000003</v>
       </c>
     </row>
@@ -97456,7 +97522,7 @@
       <c r="B275" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="C275" s="7">
+      <c r="C275">
         <v>6345.5200000000023</v>
       </c>
     </row>
@@ -97464,7 +97530,7 @@
       <c r="B276" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="C276" s="7">
+      <c r="C276">
         <v>3645.0359999999996</v>
       </c>
     </row>
@@ -97472,7 +97538,7 @@
       <c r="B277" s="6" t="s">
         <v>2121</v>
       </c>
-      <c r="C277" s="7">
+      <c r="C277">
         <v>1793.66</v>
       </c>
     </row>
@@ -97480,7 +97546,7 @@
       <c r="B278" s="6" t="s">
         <v>586</v>
       </c>
-      <c r="C278" s="7">
+      <c r="C278">
         <v>6551.6130000000012</v>
       </c>
     </row>
@@ -97488,7 +97554,7 @@
       <c r="B279" s="6" t="s">
         <v>1385</v>
       </c>
-      <c r="C279" s="7">
+      <c r="C279">
         <v>1468.9935</v>
       </c>
     </row>
@@ -97496,7 +97562,7 @@
       <c r="B280" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="C280" s="7">
+      <c r="C280">
         <v>6011.7849999999989</v>
       </c>
     </row>
@@ -97504,7 +97570,7 @@
       <c r="B281" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="C281" s="7">
+      <c r="C281">
         <v>5917.9800000000005</v>
       </c>
     </row>
@@ -97512,7 +97578,7 @@
       <c r="B282" s="6" t="s">
         <v>1442</v>
       </c>
-      <c r="C282" s="7">
+      <c r="C282">
         <v>2797.6950000000002</v>
       </c>
     </row>
@@ -97520,7 +97586,7 @@
       <c r="B283" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="C283" s="7">
+      <c r="C283">
         <v>5557.5599999999995</v>
       </c>
     </row>
@@ -97528,7 +97594,7 @@
       <c r="B284" s="6" t="s">
         <v>1953</v>
       </c>
-      <c r="C284" s="7">
+      <c r="C284">
         <v>748.79949999999997</v>
       </c>
     </row>
@@ -97536,7 +97602,7 @@
       <c r="B285" s="6" t="s">
         <v>623</v>
       </c>
-      <c r="C285" s="7">
+      <c r="C285">
         <v>1177.296</v>
       </c>
     </row>
@@ -97544,7 +97610,7 @@
       <c r="B286" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C286" s="7">
+      <c r="C286">
         <v>1403.2</v>
       </c>
     </row>
@@ -97552,7 +97618,7 @@
       <c r="B287" s="6" t="s">
         <v>789</v>
       </c>
-      <c r="C287" s="7">
+      <c r="C287">
         <v>1235.7825</v>
       </c>
     </row>
@@ -97560,7 +97626,7 @@
       <c r="B288" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="C288" s="7">
+      <c r="C288">
         <v>3610.28</v>
       </c>
     </row>
@@ -97568,7 +97634,7 @@
       <c r="B289" s="6" t="s">
         <v>1540</v>
       </c>
-      <c r="C289" s="7">
+      <c r="C289">
         <v>1812.3389999999999</v>
       </c>
     </row>
@@ -97576,7 +97642,7 @@
       <c r="B290" s="6" t="s">
         <v>832</v>
       </c>
-      <c r="C290" s="7">
+      <c r="C290">
         <v>2843.4315000000001</v>
       </c>
     </row>
@@ -97584,7 +97650,7 @@
       <c r="B291" s="6" t="s">
         <v>1447</v>
       </c>
-      <c r="C291" s="7">
+      <c r="C291">
         <v>2507.31</v>
       </c>
     </row>
@@ -97592,7 +97658,7 @@
       <c r="B292" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C292" s="7">
+      <c r="C292">
         <v>3916.8219999999988</v>
       </c>
     </row>
@@ -97600,7 +97666,7 @@
       <c r="B293" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C293" s="7">
+      <c r="C293">
         <v>3322.9559999999992</v>
       </c>
     </row>
@@ -97608,7 +97674,7 @@
       <c r="B294" s="6" t="s">
         <v>1937</v>
       </c>
-      <c r="C294" s="7">
+      <c r="C294">
         <v>763.173</v>
       </c>
     </row>
@@ -97616,7 +97682,7 @@
       <c r="B295" s="6" t="s">
         <v>1069</v>
       </c>
-      <c r="C295" s="7">
+      <c r="C295">
         <v>565.54449999999997</v>
       </c>
     </row>
@@ -97624,7 +97690,7 @@
       <c r="B296" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="C296" s="7">
+      <c r="C296">
         <v>2020.32</v>
       </c>
     </row>
@@ -97632,7 +97698,7 @@
       <c r="B297" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="C297" s="7">
+      <c r="C297">
         <v>4798.7290000000003</v>
       </c>
     </row>
@@ -97640,7 +97706,7 @@
       <c r="B298" s="6" t="s">
         <v>2138</v>
       </c>
-      <c r="C298" s="7">
+      <c r="C298">
         <v>835918.67099999986</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Perform some excel function
</commit_message>
<xml_diff>
--- a/customer_purchase_dataseet.xlsx
+++ b/customer_purchase_dataseet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Project\Fashion Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{970D09CD-A2AD-45B9-A1D7-83FBD0218A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74B2FA9D-030E-4AAC-B915-509E23FD113C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{52086F29-C266-4FF4-89C2-E090B5B922C7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{52086F29-C266-4FF4-89C2-E090B5B922C7}"/>
   </bookViews>
   <sheets>
     <sheet name="customer_purchase_dataset" sheetId="1" r:id="rId1"/>
@@ -7027,11 +7027,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -35059,7 +35059,9 @@
       <c r="O6" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P6" s="2"/>
+      <c r="P6" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -35557,7 +35559,9 @@
       <c r="O16" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P16" s="2"/>
+      <c r="P16" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
@@ -35805,7 +35809,9 @@
       <c r="O21" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P21" s="2"/>
+      <c r="P21" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
@@ -36253,7 +36259,9 @@
       <c r="O30" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P30" s="2"/>
+      <c r="P30" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
@@ -36401,7 +36409,9 @@
       <c r="O33" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P33" s="2"/>
+      <c r="P33" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
@@ -36499,7 +36509,9 @@
       <c r="O35" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P35" s="2"/>
+      <c r="P35" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
@@ -36547,7 +36559,9 @@
       <c r="O36" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P36" s="2"/>
+      <c r="P36" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
@@ -38045,7 +38059,9 @@
       <c r="O66" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P66" s="2"/>
+      <c r="P66" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
@@ -38293,7 +38309,9 @@
       <c r="O71" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P71" s="2"/>
+      <c r="P71" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
@@ -38391,7 +38409,9 @@
       <c r="O73" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P73" s="2"/>
+      <c r="P73" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
@@ -38489,7 +38509,9 @@
       <c r="O75" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P75" s="2"/>
+      <c r="P75" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
@@ -38537,7 +38559,9 @@
       <c r="O76" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P76" s="2"/>
+      <c r="P76" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
@@ -40985,7 +41009,9 @@
       <c r="O125" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P125" s="2"/>
+      <c r="P125" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
@@ -41083,7 +41109,9 @@
       <c r="O127" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P127" s="2"/>
+      <c r="P127" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="128" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
@@ -41581,7 +41609,9 @@
       <c r="O137" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P137" s="2"/>
+      <c r="P137" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="138" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
@@ -42179,7 +42209,9 @@
       <c r="O149" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P149" s="2"/>
+      <c r="P149" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="150" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
@@ -42527,7 +42559,9 @@
       <c r="O156" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P156" s="2"/>
+      <c r="P156" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="157" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
@@ -43125,7 +43159,9 @@
       <c r="O168" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P168" s="2"/>
+      <c r="P168" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="169" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
@@ -43323,7 +43359,9 @@
       <c r="O172" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P172" s="2"/>
+      <c r="P172" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="173" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
@@ -43371,7 +43409,9 @@
       <c r="O173" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P173" s="2"/>
+      <c r="P173" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="174" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
@@ -43669,7 +43709,9 @@
       <c r="O179" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P179" s="2"/>
+      <c r="P179" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="180" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
@@ -44017,7 +44059,9 @@
       <c r="O186" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P186" s="2"/>
+      <c r="P186" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="187" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
@@ -45015,7 +45059,9 @@
       <c r="O206" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P206" s="2"/>
+      <c r="P206" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="207" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
@@ -45413,7 +45459,9 @@
       <c r="O214" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P214" s="2"/>
+      <c r="P214" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="215" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
@@ -45661,7 +45709,9 @@
       <c r="O219" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P219" s="2"/>
+      <c r="P219" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="220" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A220" s="2" t="s">
@@ -46409,7 +46459,9 @@
       <c r="O234" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P234" s="2"/>
+      <c r="P234" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="235" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A235" s="2" t="s">
@@ -46557,7 +46609,9 @@
       <c r="O237" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P237" s="2"/>
+      <c r="P237" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="238" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A238" s="2" t="s">
@@ -47505,7 +47559,9 @@
       <c r="O256" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P256" s="2"/>
+      <c r="P256" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="257" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A257" s="2" t="s">
@@ -47803,7 +47859,9 @@
       <c r="O262" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P262" s="2"/>
+      <c r="P262" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="263" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A263" s="2" t="s">
@@ -47851,7 +47909,9 @@
       <c r="O263" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P263" s="2"/>
+      <c r="P263" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="264" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A264" s="2" t="s">
@@ -47899,7 +47959,9 @@
       <c r="O264" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P264" s="2"/>
+      <c r="P264" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="265" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A265" s="2" t="s">
@@ -48247,7 +48309,9 @@
       <c r="O271" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P271" s="2"/>
+      <c r="P271" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="272" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A272" s="2" t="s">
@@ -48445,7 +48509,9 @@
       <c r="O275" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P275" s="2"/>
+      <c r="P275" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="276" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A276" s="2" t="s">
@@ -48493,7 +48559,9 @@
       <c r="O276" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P276" s="2"/>
+      <c r="P276" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="277" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A277" s="2" t="s">
@@ -50291,7 +50359,9 @@
       <c r="O312" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P312" s="2"/>
+      <c r="P312" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="313" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A313" s="2" t="s">
@@ -51039,7 +51109,9 @@
       <c r="O327" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P327" s="2"/>
+      <c r="P327" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="328" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A328" s="2" t="s">
@@ -51187,7 +51259,9 @@
       <c r="O330" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P330" s="2"/>
+      <c r="P330" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="331" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A331" s="2" t="s">
@@ -51685,7 +51759,9 @@
       <c r="O340" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P340" s="2"/>
+      <c r="P340" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="341" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A341" s="2" t="s">
@@ -51733,7 +51809,9 @@
       <c r="O341" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P341" s="2"/>
+      <c r="P341" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="342" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A342" s="2" t="s">
@@ -52831,7 +52909,9 @@
       <c r="O363" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P363" s="2"/>
+      <c r="P363" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="364" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A364" s="2" t="s">
@@ -53029,7 +53109,9 @@
       <c r="O367" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P367" s="2"/>
+      <c r="P367" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="368" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A368" s="2" t="s">
@@ -53227,7 +53309,9 @@
       <c r="O371" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P371" s="2"/>
+      <c r="P371" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="372" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A372" s="2" t="s">
@@ -54375,7 +54459,9 @@
       <c r="O394" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P394" s="2"/>
+      <c r="P394" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="395" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A395" s="2" t="s">
@@ -54773,7 +54859,9 @@
       <c r="O402" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P402" s="2"/>
+      <c r="P402" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="403" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A403" s="2" t="s">
@@ -55121,7 +55209,9 @@
       <c r="O409" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P409" s="2"/>
+      <c r="P409" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="410" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A410" s="2" t="s">
@@ -55319,7 +55409,9 @@
       <c r="O413" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P413" s="2"/>
+      <c r="P413" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="414" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A414" s="2" t="s">
@@ -55967,7 +56059,9 @@
       <c r="O426" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P426" s="2"/>
+      <c r="P426" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="427" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A427" s="2" t="s">
@@ -56015,7 +56109,9 @@
       <c r="O427" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P427" s="2"/>
+      <c r="P427" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="428" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A428" s="2" t="s">
@@ -56113,7 +56209,9 @@
       <c r="O429" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P429" s="2"/>
+      <c r="P429" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="430" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A430" s="2" t="s">
@@ -56961,7 +57059,9 @@
       <c r="O446" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P446" s="2"/>
+      <c r="P446" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="447" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A447" s="2" t="s">
@@ -57009,7 +57109,9 @@
       <c r="O447" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P447" s="2"/>
+      <c r="P447" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="448" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A448" s="2" t="s">
@@ -57157,7 +57259,9 @@
       <c r="O450" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P450" s="2"/>
+      <c r="P450" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="451" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A451" s="2" t="s">
@@ -57805,7 +57909,9 @@
       <c r="O463" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P463" s="2"/>
+      <c r="P463" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="464" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A464" s="2" t="s">
@@ -57903,7 +58009,9 @@
       <c r="O465" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P465" s="2"/>
+      <c r="P465" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="466" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A466" s="2" t="s">
@@ -57951,7 +58059,9 @@
       <c r="O466" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P466" s="2"/>
+      <c r="P466" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="467" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A467" s="2" t="s">
@@ -58449,7 +58559,9 @@
       <c r="O476" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P476" s="2"/>
+      <c r="P476" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="477" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A477" s="2" t="s">
@@ -59997,7 +60109,9 @@
       <c r="O507" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P507" s="2"/>
+      <c r="P507" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="508" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A508" s="2" t="s">
@@ -60495,7 +60609,9 @@
       <c r="O517" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P517" s="2"/>
+      <c r="P517" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="518" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A518" s="2" t="s">
@@ -61043,7 +61159,9 @@
       <c r="O528" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P528" s="2"/>
+      <c r="P528" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="529" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A529" s="2" t="s">
@@ -61241,7 +61359,9 @@
       <c r="O532" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P532" s="2"/>
+      <c r="P532" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="533" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A533" s="2" t="s">
@@ -61289,7 +61409,9 @@
       <c r="O533" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P533" s="2"/>
+      <c r="P533" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="534" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A534" s="2" t="s">
@@ -62337,7 +62459,9 @@
       <c r="O554" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P554" s="2"/>
+      <c r="P554" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="555" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A555" s="2" t="s">
@@ -63685,7 +63809,9 @@
       <c r="O581" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P581" s="2"/>
+      <c r="P581" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="582" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A582" s="2" t="s">
@@ -64083,7 +64209,9 @@
       <c r="O589" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P589" s="2"/>
+      <c r="P589" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="590" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A590" s="2" t="s">
@@ -64381,7 +64509,9 @@
       <c r="O595" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P595" s="2"/>
+      <c r="P595" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="596" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A596" s="2" t="s">
@@ -64879,7 +65009,9 @@
       <c r="O605" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P605" s="2"/>
+      <c r="P605" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="606" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A606" s="2" t="s">
@@ -65827,7 +65959,9 @@
       <c r="O624" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P624" s="2"/>
+      <c r="P624" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="625" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A625" s="2" t="s">
@@ -66925,7 +67059,9 @@
       <c r="O646" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P646" s="2"/>
+      <c r="P646" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="647" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A647" s="2" t="s">
@@ -67173,7 +67309,9 @@
       <c r="O651" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P651" s="2"/>
+      <c r="P651" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="652" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A652" s="2" t="s">
@@ -67571,7 +67709,9 @@
       <c r="O659" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P659" s="2"/>
+      <c r="P659" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="660" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A660" s="2" t="s">
@@ -69269,7 +69409,9 @@
       <c r="O693" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P693" s="2"/>
+      <c r="P693" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="694" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A694" s="2" t="s">
@@ -69667,7 +69809,9 @@
       <c r="O701" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P701" s="2"/>
+      <c r="P701" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="702" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A702" s="2" t="s">
@@ -70615,7 +70759,9 @@
       <c r="O720" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P720" s="2"/>
+      <c r="P720" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="721" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A721" s="2" t="s">
@@ -70763,7 +70909,9 @@
       <c r="O723" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P723" s="2"/>
+      <c r="P723" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="724" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A724" s="2" t="s">
@@ -71111,7 +71259,9 @@
       <c r="O730" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P730" s="2"/>
+      <c r="P730" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="731" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A731" s="2" t="s">
@@ -71459,7 +71609,9 @@
       <c r="O737" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P737" s="2"/>
+      <c r="P737" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="738" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A738" s="2" t="s">
@@ -72607,7 +72759,9 @@
       <c r="O760" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P760" s="2"/>
+      <c r="P760" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="761" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A761" s="2" t="s">
@@ -72905,7 +73059,9 @@
       <c r="O766" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P766" s="2"/>
+      <c r="P766" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="767" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A767" s="2" t="s">
@@ -73503,7 +73659,9 @@
       <c r="O778" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P778" s="2"/>
+      <c r="P778" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="779" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A779" s="2" t="s">
@@ -73701,7 +73859,9 @@
       <c r="O782" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P782" s="2"/>
+      <c r="P782" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="783" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A783" s="2" t="s">
@@ -74149,7 +74309,9 @@
       <c r="O791" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P791" s="2"/>
+      <c r="P791" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="792" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A792" s="2" t="s">
@@ -75047,7 +75209,9 @@
       <c r="O809" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P809" s="2"/>
+      <c r="P809" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="810" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A810" s="2" t="s">
@@ -75245,7 +75409,9 @@
       <c r="O813" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P813" s="2"/>
+      <c r="P813" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="814" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A814" s="2" t="s">
@@ -75843,7 +76009,9 @@
       <c r="O825" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P825" s="2"/>
+      <c r="P825" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="826" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A826" s="2" t="s">
@@ -75941,7 +76109,9 @@
       <c r="O827" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P827" s="2"/>
+      <c r="P827" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="828" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A828" s="2" t="s">
@@ -77689,7 +77859,9 @@
       <c r="O862" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P862" s="2"/>
+      <c r="P862" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="863" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A863" s="2" t="s">
@@ -78087,7 +78259,9 @@
       <c r="O870" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P870" s="2"/>
+      <c r="P870" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="871" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A871" s="2" t="s">
@@ -78535,7 +78709,9 @@
       <c r="O879" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P879" s="2"/>
+      <c r="P879" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="880" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A880" s="2" t="s">
@@ -79333,7 +79509,9 @@
       <c r="O895" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P895" s="2"/>
+      <c r="P895" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="896" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A896" s="2" t="s">
@@ -81281,7 +81459,9 @@
       <c r="O934" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P934" s="2"/>
+      <c r="P934" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="935" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A935" s="2" t="s">
@@ -81429,7 +81609,9 @@
       <c r="O937" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P937" s="2"/>
+      <c r="P937" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="938" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A938" s="2" t="s">
@@ -82577,7 +82759,9 @@
       <c r="O960" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P960" s="2"/>
+      <c r="P960" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="961" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A961" s="2" t="s">
@@ -82725,7 +82909,9 @@
       <c r="O963" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P963" s="2"/>
+      <c r="P963" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="964" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A964" s="2" t="s">
@@ -83723,7 +83909,9 @@
       <c r="O983" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P983" s="2"/>
+      <c r="P983" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="984" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A984" s="2" t="s">
@@ -84621,7 +84809,9 @@
       <c r="O1001" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1001" s="2"/>
+      <c r="P1001" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1002" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1002" s="2" t="s">
@@ -84719,7 +84909,9 @@
       <c r="O1003" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P1003" s="2"/>
+      <c r="P1003" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1004" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1004" s="2" t="s">
@@ -85267,7 +85459,9 @@
       <c r="O1014" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1014" s="2"/>
+      <c r="P1014" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1015" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1015" s="2" t="s">
@@ -85865,7 +86059,9 @@
       <c r="O1026" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1026" s="2"/>
+      <c r="P1026" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1027" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1027" s="2" t="s">
@@ -86463,7 +86659,9 @@
       <c r="O1038" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1038" s="2"/>
+      <c r="P1038" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1039" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1039" s="2" t="s">
@@ -86511,7 +86709,9 @@
       <c r="O1039" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1039" s="2"/>
+      <c r="P1039" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1040" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1040" s="2" t="s">
@@ -87209,7 +87409,9 @@
       <c r="O1053" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1053" s="2"/>
+      <c r="P1053" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1054" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1054" s="2" t="s">
@@ -87507,7 +87709,9 @@
       <c r="O1059" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P1059" s="2"/>
+      <c r="P1059" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1060" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1060" s="2" t="s">
@@ -89355,7 +89559,9 @@
       <c r="O1096" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P1096" s="2"/>
+      <c r="P1096" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1097" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1097" s="2" t="s">
@@ -89503,7 +89709,9 @@
       <c r="O1099" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1099" s="2"/>
+      <c r="P1099" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1100" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1100" s="2" t="s">
@@ -90151,7 +90359,9 @@
       <c r="O1112" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P1112" s="2"/>
+      <c r="P1112" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1113" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1113" s="2" t="s">
@@ -90599,7 +90809,9 @@
       <c r="O1121" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P1121" s="2"/>
+      <c r="P1121" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1122" s="2" t="s">
@@ -90647,7 +90859,9 @@
       <c r="O1122" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P1122" s="2"/>
+      <c r="P1122" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1123" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1123" s="2" t="s">
@@ -90795,7 +91009,9 @@
       <c r="O1125" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P1125" s="2"/>
+      <c r="P1125" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1126" s="2" t="s">
@@ -91493,7 +91709,9 @@
       <c r="O1139" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P1139" s="2"/>
+      <c r="P1139" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1140" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1140" s="2" t="s">
@@ -91841,7 +92059,9 @@
       <c r="O1146" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P1146" s="2"/>
+      <c r="P1146" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1147" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1147" s="2" t="s">
@@ -91939,7 +92159,9 @@
       <c r="O1148" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P1148" s="2"/>
+      <c r="P1148" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1149" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1149" s="2" t="s">
@@ -92237,7 +92459,9 @@
       <c r="O1154" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P1154" s="2"/>
+      <c r="P1154" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1155" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1155" s="2" t="s">
@@ -92535,7 +92759,9 @@
       <c r="O1160" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1160" s="2"/>
+      <c r="P1160" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1161" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1161" s="2" t="s">
@@ -93483,7 +93709,9 @@
       <c r="O1179" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P1179" s="2"/>
+      <c r="P1179" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1180" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1180" s="2" t="s">
@@ -93781,7 +94009,9 @@
       <c r="O1185" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1185" s="2"/>
+      <c r="P1185" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1186" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1186" s="2" t="s">
@@ -94079,7 +94309,9 @@
       <c r="O1191" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P1191" s="2"/>
+      <c r="P1191" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1192" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1192" s="2" t="s">
@@ -94127,7 +94359,9 @@
       <c r="O1192" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1192" s="2"/>
+      <c r="P1192" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1193" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1193" s="2" t="s">
@@ -94225,7 +94459,9 @@
       <c r="O1194" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P1194" s="2"/>
+      <c r="P1194" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="1195" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1195" s="2" t="s">
@@ -94719,12 +94955,12 @@
       <c r="W3" s="1" t="s">
         <v>2143</v>
       </c>
-      <c r="Y3" s="7" t="s">
+      <c r="Y3" s="9" t="s">
         <v>2144</v>
       </c>
-      <c r="Z3" s="7"/>
-      <c r="AA3" s="7"/>
-      <c r="AB3" s="7"/>
+      <c r="Z3" s="9"/>
+      <c r="AA3" s="9"/>
+      <c r="AB3" s="9"/>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -94786,18 +95022,18 @@
       </c>
       <c r="W4" s="4">
         <f>ROUND(AVERAGE(customer_purchase_dataset!P2:P1201),2)</f>
-        <v>3.58</v>
-      </c>
-      <c r="Y4" s="8" t="s">
+        <v>3.22</v>
+      </c>
+      <c r="Y4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="Z4" s="8" t="s">
+      <c r="Z4" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="AA4" s="8" t="s">
+      <c r="AA4" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="AB4" s="8" t="s">
+      <c r="AB4" s="7" t="s">
         <v>24</v>
       </c>
     </row>
@@ -94851,17 +95087,17 @@
       <c r="P5" s="4">
         <v>5</v>
       </c>
-      <c r="Y5" s="9" cm="1">
+      <c r="Y5" s="8" cm="1">
         <f t="array" ref="Y5:AB5">COUNTIFS(customer_purchase_dataset!O2:O1201,Summery!Y4:AB4)</f>
         <v>694</v>
       </c>
-      <c r="Z5" s="9">
+      <c r="Z5" s="8">
         <v>180</v>
       </c>
-      <c r="AA5" s="9">
+      <c r="AA5" s="8">
         <v>158</v>
       </c>
-      <c r="AB5" s="9">
+      <c r="AB5" s="8">
         <v>168</v>
       </c>
     </row>

</xml_diff>